<commit_message>
docs: questionnaire 7 — end of the kayak text, lighthouse photo without watermark, Enclaves bridge struck on Franck's capture; dropdown choices without commas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/questions-kibreeze-franck-7.xlsx
+++ b/docs/questions-kibreeze-franck-7.xlsx
@@ -369,1464 +369,1514 @@
       <row>10</row>
       <rowOff>0</rowOff>
     </from>
+    <ext cx="714375" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
     <ext cx="733425" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="6" name="Image 6" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId6"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>12</row>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>13</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="714375" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="7" name="Image 7" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId7"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>14</row>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>15</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="714375" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="8" name="Image 8" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId8"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>16</row>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="733425" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="9" name="Image 9" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId9"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>18</row>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>19</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="714375" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="10" name="Image 10" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId10"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>19</row>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="714375" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="11" name="Image 11" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId11"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>20</row>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>21</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="714375" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="12" name="Image 12" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId12"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>21</row>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>22</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="590550" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="13" name="Image 13" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId13"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>22</row>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>23</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="590550" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="14" name="Image 14" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId14"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>23</row>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>24</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="590550" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="15" name="Image 15" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId15"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>24</row>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>25</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="714375" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="16" name="Image 16" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId16"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>25</row>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>26</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="590550" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="17" name="Image 17" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId17"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>26</row>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>27</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1266825" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="18" name="Image 18" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId18"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>28</row>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>29</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="714375" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="19" name="Image 19" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId19"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>29</row>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>30</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="714375" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="20" name="Image 20" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId20"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>30</row>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId21"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>31</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="981075" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="21" name="Image 21" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId21"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>31</row>
+        <cNvPr id="22" name="Image 22" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId22"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>32</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="952500" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="22" name="Image 22" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId22"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>32</row>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId23"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>33</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="638175" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="23" name="Image 23" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId23"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>33</row>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId24"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>34</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="714375" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="24" name="Image 24" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId24"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>34</row>
+        <cNvPr id="25" name="Image 25" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId25"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>35</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1266825" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="25" name="Image 25" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId25"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>35</row>
+        <cNvPr id="26" name="Image 26" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId26"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>36</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1276350" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="26" name="Image 26" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId26"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>36</row>
+        <cNvPr id="27" name="Image 27" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId27"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>37</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="714375" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="27" name="Image 27" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId27"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>37</row>
+        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId28"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>38</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="533400" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="28" name="Image 28" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId28"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>38</row>
+        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId29"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>39</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1428750" cy="752475"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="29" name="Image 29" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId29"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>39</row>
+        <cNvPr id="30" name="Image 30" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId30"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>40</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="714375" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="30" name="Image 30" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId30"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>40</row>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId31"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>41</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1428750" cy="800100"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="31" name="Image 31" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId31"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>42</row>
+        <cNvPr id="32" name="Image 32" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId32"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>43</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1276350" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="32" name="Image 32" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId32"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>43</row>
+        <cNvPr id="33" name="Image 33" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId33"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>44</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1276350" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="33" name="Image 33" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId33"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>44</row>
+        <cNvPr id="34" name="Image 34" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId34"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>45</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1276350" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="34" name="Image 34" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId34"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>45</row>
+        <cNvPr id="35" name="Image 35" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId35"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>46</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1276350" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="35" name="Image 35" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId35"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>46</row>
+        <cNvPr id="36" name="Image 36" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId36"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>47</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1276350" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="36" name="Image 36" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId36"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>47</row>
+        <cNvPr id="37" name="Image 37" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId37"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>48</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="38" name="Image 38" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId38"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>49</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="39" name="Image 39" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId39"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>50</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1276350" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="37" name="Image 37" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId37"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>48</row>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId40"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>51</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1276350" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="38" name="Image 38" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId38"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>49</row>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId41"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>52</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1276350" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="39" name="Image 39" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId39"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>50</row>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId42"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>53</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1276350" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="40" name="Image 40" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId40"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>51</row>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId43"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>55</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="44" name="Image 44" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId44"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>56</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="45" name="Image 45" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId45"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>57</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="46" name="Image 46" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId46"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>58</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="590550" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="47" name="Image 47" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId47"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>59</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="48" name="Image 48" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId48"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>60</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1266825" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="49" name="Image 49" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId49"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>62</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1266825" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="50" name="Image 50" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId50"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>63</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="638175" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="51" name="Image 51" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId51"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>64</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="52" name="Image 52" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId52"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>65</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1276350" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="41" name="Image 41" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId41"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>53</row>
+        <cNvPr id="53" name="Image 53" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId53"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>67</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="800100"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="54" name="Image 54" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId54"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>68</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="800100"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="55" name="Image 55" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId55"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>69</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="800100"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="56" name="Image 56" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId56"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>70</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="800100"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="57" name="Image 57" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId57"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>71</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="800100"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="58" name="Image 58" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId58"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>72</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="800100"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="59" name="Image 59" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId59"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>74</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="714375" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="42" name="Image 42" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId42"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>54</row>
+        <cNvPr id="60" name="Image 60" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId60"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>75</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="714375" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="43" name="Image 43" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId43"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>55</row>
+        <cNvPr id="61" name="Image 61" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId61"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>76</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1285875" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="62" name="Image 62" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId62"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>77</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="714375" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="44" name="Image 44" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId44"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>56</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="590550" cy="952500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="45" name="Image 45" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId45"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>57</row>
+        <cNvPr id="63" name="Image 63" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId63"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>78</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="714375" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="46" name="Image 46" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId46"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>58</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1266825" cy="952500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="47" name="Image 47" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId47"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>60</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1266825" cy="952500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="48" name="Image 48" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId48"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>61</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="638175" cy="952500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="49" name="Image 49" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId49"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>62</row>
+        <cNvPr id="64" name="Image 64" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId64"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>79</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="714375" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="50" name="Image 50" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId50"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>63</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1276350" cy="952500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="51" name="Image 51" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId51"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>65</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1428750" cy="800100"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="52" name="Image 52" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId52"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>66</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1428750" cy="800100"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="53" name="Image 53" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId53"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>67</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1428750" cy="800100"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="54" name="Image 54" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId54"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>68</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1428750" cy="800100"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="55" name="Image 55" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId55"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>69</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1428750" cy="800100"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="56" name="Image 56" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId56"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>70</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1428750" cy="800100"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="57" name="Image 57" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId57"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>72</row>
+        <cNvPr id="65" name="Image 65" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId65"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>80</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="714375" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="58" name="Image 58" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId58"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>73</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="714375" cy="952500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="59" name="Image 59" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId59"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>74</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1285875" cy="952500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="60" name="Image 60" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId60"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>75</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="714375" cy="952500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="61" name="Image 61" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId61"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>76</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="714375" cy="952500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="62" name="Image 62" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId62"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>77</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="714375" cy="952500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="63" name="Image 63" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId63"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>78</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="714375" cy="952500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="64" name="Image 64" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId64"/>
+        <cNvPr id="66" name="Image 66" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId66"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2139,21 +2189,21 @@
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Kibreeze — tes retours des 11 et 12 octobre</t>
+          <t>Kibreeze — tes retours des 11, 12 et 18 octobre</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Questions de Zobel   |   18 octobre 2026</t>
+          <t>Questions de Zobel   |   19 octobre 2026</t>
         </is>
       </c>
     </row>
     <row r="4" ht="56" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Franck, merci pour tes retours sur le site. On a tout repris : les plats se comptent maintenant en « plats », tes descriptions et l'Ebanjea sont intégrés, chaque parcours aura sa fiche avec sa durée, les dates se choisiront dans un calendrier, et l'accueil aura un diaporama et un aperçu des véhicules. Pour finir, il me manque quelques informations de toi.</t>
+          <t>Franck, merci pour tes retours sur le site. On a tout repris : les plats se comptent maintenant en « plats », tes descriptions et l'Ebanjea sont intégrés, chaque parcours aura sa fiche avec sa durée, les dates se choisissent dans un calendrier, l'accueil a un diaporama et un aperçu des véhicules, tes descriptions des activités et des parcours sont en ligne, et dans Mon séjour le nombre de personnes se règle une seule fois (« Voyageurs »), chaque ligne n'ayant plus qu'un compteur de sessions. Pour finir, il me manque quelques informations de toi.</t>
         </is>
       </c>
     </row>
@@ -2178,10 +2228,10 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="28" customHeight="1">
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>1. Questions : prix par personne pour la pirogue, la chaloupe et le feu de plage ; tes liens WhatsApp ; le maban et l'Ebanjea.</t>
+          <t>1. Questions : prix par personne pour la pirogue, la chaloupe et le feu de plage ; tes liens WhatsApp ; le maban et l'Ebanjea ; la fin du texte du kayak ; le phare et le pont des Enclaves du village Mayi.</t>
         </is>
       </c>
     </row>
@@ -2210,7 +2260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2225,7 +2275,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Questions : 7 points</t>
+          <t>Questions : 10 points</t>
         </is>
       </c>
     </row>
@@ -2407,12 +2457,12 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>Oui, garde ce numéro  /  Autre numéro (précise)</t>
+          <t>Garder ce numéro  /  Autre numéro (précise)</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
-          <t>Oui, garde ce numéro</t>
+          <t>Garder ce numéro</t>
         </is>
       </c>
       <c r="F9" s="11" t="n"/>
@@ -2476,8 +2526,95 @@
       <c r="F11" s="11" t="n"/>
       <c r="G11" s="11" t="n"/>
     </row>
+    <row r="12" ht="80" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Kayak : fin du texte</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Ton texte du kayak est arrivé coupé : « …dans une ambiance apaisante où chaque coup de pagaie devient une invitation à ». En attendant, le site s'arrête à « …dans une ambiance apaisante. » Écris-moi la fin de la phrase.</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Réponse libre</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>…devient une invitation à la détente.</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
+    </row>
+    <row r="13" ht="80" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Q9</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Village Mayi : photo du phare</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>La fiche du village Mayi n'a pas de photo du phare. Les trois photos du phare de tes envois (L13-02, L13-03, L13-04) portent un filigrane : on ne peut pas les publier. Peux-tu m'en envoyer une sans filigrane ?</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Je t'envoie une photo  /  Pas de photo du phare pour le moment</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Je t'envoie une photo</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="n"/>
+      <c r="G13" s="11" t="n"/>
+    </row>
+    <row r="14" ht="80" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Q10</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Village Mayi : pont des Enclaves</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Sur ta capture de la carte du village Mayi, « le pont des Enclaves » est barré d'un trait vert. Le 18 octobre, tu avais écrit « ponts de l'Esclavage et des Enclaves ». Faut-il le retirer de la description ?</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Le retirer  /  Le garder (trait involontaire)  /  Autre (précise)</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Le garder (trait involontaire)</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="n"/>
+      <c r="G14" s="11" t="n"/>
+    </row>
   </sheetData>
-  <dataValidations count="6">
+  <dataValidations count="8">
     <dataValidation sqref="F5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Prix par personne (précise),Garder seulement le prix groupe"</formula1>
     </dataValidation>
@@ -2488,13 +2625,19 @@
       <formula1>"Prix par personne (précise),Garder seulement le prix groupe"</formula1>
     </dataValidation>
     <dataValidation sqref="F9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Oui, garde ce numéro,Autre numéro (précise)"</formula1>
+      <formula1>"Garder ce numéro,Autre numéro (précise)"</formula1>
     </dataValidation>
     <dataValidation sqref="F10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Je t'envoie une photo,Je te le décris (précise)"</formula1>
     </dataValidation>
     <dataValidation sqref="F11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Je t'envoie une photo,Je te le décris (précise)"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Je t'envoie une photo,Pas de photo du phare pour le moment"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Le retirer,Le garder (trait involontaire),Autre (précise)"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2507,7 +2650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G79"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2522,7 +2665,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Photos : 64 emplacements</t>
+          <t>Photos : 66 emplacements</t>
         </is>
       </c>
     </row>
@@ -2696,154 +2839,154 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Aperçu hébergement : Villa</t>
+          <t>Aperçu hébergement : Appartement</t>
         </is>
       </c>
       <c r="C11" s="9" t="n"/>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>accommodation/villa.jpg</t>
+          <t>accommodation/appartement.jpg</t>
         </is>
       </c>
       <c r="E11" s="11" t="n"/>
       <c r="F11" s="11" t="n"/>
       <c r="G11" s="11" t="n"/>
     </row>
-    <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+    <row r="12" ht="80" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Accueil</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Aperçu hébergement : Villa</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>accommodation/villa.jpg</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Contact</t>
         </is>
       </c>
-      <c r="B12" s="13" t="n"/>
-      <c r="C12" s="13" t="n"/>
-      <c r="D12" s="13" t="n"/>
-      <c r="E12" s="13" t="n"/>
-      <c r="F12" s="13" t="n"/>
-      <c r="G12" s="13" t="n"/>
-    </row>
-    <row r="13" ht="80" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="B13" s="13" t="n"/>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="13" t="n"/>
+      <c r="E13" s="13" t="n"/>
+      <c r="F13" s="13" t="n"/>
+      <c r="G13" s="13" t="n"/>
+    </row>
+    <row r="14" ht="80" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Contact</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Qui sommes-nous</t>
         </is>
       </c>
-      <c r="C13" s="9" t="n"/>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="C14" s="9" t="n"/>
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>sections/plage-kribi.jpg</t>
         </is>
       </c>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+      <c r="G14" s="11" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>Tourisme</t>
         </is>
       </c>
-      <c r="B14" s="13" t="n"/>
-      <c r="C14" s="13" t="n"/>
-      <c r="D14" s="13" t="n"/>
-      <c r="E14" s="13" t="n"/>
-      <c r="F14" s="13" t="n"/>
-      <c r="G14" s="13" t="n"/>
-    </row>
-    <row r="15" ht="80" customHeight="1">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="B15" s="13" t="n"/>
+      <c r="C15" s="13" t="n"/>
+      <c r="D15" s="13" t="n"/>
+      <c r="E15" s="13" t="n"/>
+      <c r="F15" s="13" t="n"/>
+      <c r="G15" s="13" t="n"/>
+    </row>
+    <row r="16" ht="80" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>Tourisme</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Bandeau de la page Tourisme</t>
         </is>
       </c>
-      <c r="C15" s="9" t="n"/>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="C16" s="9" t="n"/>
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>sections/bandeau-experiences.jpg</t>
         </is>
       </c>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="11" t="n"/>
-      <c r="G15" s="11" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>Hébergements</t>
         </is>
       </c>
-      <c r="B16" s="13" t="n"/>
-      <c r="C16" s="13" t="n"/>
-      <c r="D16" s="13" t="n"/>
-      <c r="E16" s="13" t="n"/>
-      <c r="F16" s="13" t="n"/>
-      <c r="G16" s="13" t="n"/>
-    </row>
-    <row r="17" ht="80" customHeight="1">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="B17" s="13" t="n"/>
+      <c r="C17" s="13" t="n"/>
+      <c r="D17" s="13" t="n"/>
+      <c r="E17" s="13" t="n"/>
+      <c r="F17" s="13" t="n"/>
+      <c r="G17" s="13" t="n"/>
+    </row>
+    <row r="18" ht="80" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>Hébergements</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Bandeau de la page Hébergements</t>
         </is>
       </c>
-      <c r="C17" s="9" t="n"/>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="C18" s="9" t="n"/>
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>accommodation/villa.jpg</t>
         </is>
       </c>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="11" t="n"/>
-      <c r="G17" s="11" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>Tourisme — Visites &amp; Découvertes</t>
         </is>
       </c>
-      <c r="B18" s="13" t="n"/>
-      <c r="C18" s="13" t="n"/>
-      <c r="D18" s="13" t="n"/>
-      <c r="E18" s="13" t="n"/>
-      <c r="F18" s="13" t="n"/>
-      <c r="G18" s="13" t="n"/>
-    </row>
-    <row r="19" ht="80" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>Tourisme — Visites &amp; Découvertes</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>Chutes de la Lobé (+2 photos)</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>experiences/chutes-de-la-lobe.jpg</t>
-        </is>
-      </c>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="11" t="n"/>
-      <c r="G19" s="11" t="n"/>
+      <c r="B19" s="13" t="n"/>
+      <c r="C19" s="13" t="n"/>
+      <c r="D19" s="13" t="n"/>
+      <c r="E19" s="13" t="n"/>
+      <c r="F19" s="13" t="n"/>
+      <c r="G19" s="13" t="n"/>
     </row>
     <row r="20" ht="80" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
@@ -2853,13 +2996,13 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Village Bagyeli (+2 photos)</t>
+          <t>Chutes de la Lobé (+2 photos)</t>
         </is>
       </c>
       <c r="C20" s="9" t="n"/>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>experiences/campement-bagyeli.jpg</t>
+          <t>experiences/chutes-de-la-lobe.jpg</t>
         </is>
       </c>
       <c r="E20" s="11" t="n"/>
@@ -2874,13 +3017,13 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Village Mayi (+1 photo)</t>
+          <t>Village Bagyeli (+2 photos)</t>
         </is>
       </c>
       <c r="C21" s="9" t="n"/>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>experiences/village-mayi.jpg</t>
+          <t>experiences/campement-bagyeli.jpg</t>
         </is>
       </c>
       <c r="E21" s="11" t="n"/>
@@ -2895,13 +3038,13 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Village Ebodjé et tortues marines</t>
+          <t>Village Mayi (+1 photo)</t>
         </is>
       </c>
       <c r="C22" s="9" t="n"/>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>sections/kribi-vue-aerienne.jpg</t>
+          <t>experiences/village-mayi.jpg</t>
         </is>
       </c>
       <c r="E22" s="11" t="n"/>
@@ -2916,7 +3059,7 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Port Autonome de Kribi</t>
+          <t>Village Ebodjé et tortues marines</t>
         </is>
       </c>
       <c r="C23" s="9" t="n"/>
@@ -2937,7 +3080,7 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Hôtel Golden K, visite</t>
+          <t>Port Autonome de Kribi</t>
         </is>
       </c>
       <c r="C24" s="9" t="n"/>
@@ -2958,13 +3101,13 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Plage du village Batanga</t>
+          <t>Hôtel Golden K, visite</t>
         </is>
       </c>
       <c r="C25" s="9" t="n"/>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>experiences/plage-de-batanga.jpg</t>
+          <t>sections/kribi-vue-aerienne.jpg</t>
         </is>
       </c>
       <c r="E25" s="11" t="n"/>
@@ -2979,13 +3122,13 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Musée Batanga</t>
+          <t>Plage du village Batanga</t>
         </is>
       </c>
       <c r="C26" s="9" t="n"/>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>sections/kribi-vue-aerienne.jpg</t>
+          <t>experiences/plage-de-batanga.jpg</t>
         </is>
       </c>
       <c r="E26" s="11" t="n"/>
@@ -3000,52 +3143,52 @@
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Débarcadère de Mboa-Manga</t>
+          <t>Musée Batanga</t>
         </is>
       </c>
       <c r="C27" s="9" t="n"/>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>experiences/debarcadere-de-mboa-manga.jpg</t>
+          <t>sections/kribi-vue-aerienne.jpg</t>
         </is>
       </c>
       <c r="E27" s="11" t="n"/>
       <c r="F27" s="11" t="n"/>
       <c r="G27" s="11" t="n"/>
     </row>
-    <row r="28">
-      <c r="A28" s="12" t="inlineStr">
+    <row r="28" ht="80" customHeight="1">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>Tourisme — Visites &amp; Découvertes</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Débarcadère de Mboa-Manga</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="n"/>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>experiences/debarcadere-de-mboa-manga.jpg</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="n"/>
+      <c r="F28" s="11" t="n"/>
+      <c r="G28" s="11" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
         <is>
           <t>Tourisme — Activités &amp; Loisirs</t>
         </is>
       </c>
-      <c r="B28" s="13" t="n"/>
-      <c r="C28" s="13" t="n"/>
-      <c r="D28" s="13" t="n"/>
-      <c r="E28" s="13" t="n"/>
-      <c r="F28" s="13" t="n"/>
-      <c r="G28" s="13" t="n"/>
-    </row>
-    <row r="29" ht="80" customHeight="1">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>Tourisme — Activités &amp; Loisirs</t>
-        </is>
-      </c>
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t>Quad (+2 photos)</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="n"/>
-      <c r="D29" s="9" t="inlineStr">
-        <is>
-          <t>experiences/quad.jpg</t>
-        </is>
-      </c>
-      <c r="E29" s="11" t="n"/>
-      <c r="F29" s="11" t="n"/>
-      <c r="G29" s="11" t="n"/>
+      <c r="B29" s="13" t="n"/>
+      <c r="C29" s="13" t="n"/>
+      <c r="D29" s="13" t="n"/>
+      <c r="E29" s="13" t="n"/>
+      <c r="F29" s="13" t="n"/>
+      <c r="G29" s="13" t="n"/>
     </row>
     <row r="30" ht="80" customHeight="1">
       <c r="A30" s="9" t="inlineStr">
@@ -3055,13 +3198,13 @@
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>Jet-ski (+2 photos)</t>
+          <t>Quad (+2 photos)</t>
         </is>
       </c>
       <c r="C30" s="9" t="n"/>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>experiences/jet-ski.jpg</t>
+          <t>experiences/quad.jpg</t>
         </is>
       </c>
       <c r="E30" s="11" t="n"/>
@@ -3076,13 +3219,13 @@
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Kayak</t>
+          <t>Jet-ski (+2 photos)</t>
         </is>
       </c>
       <c r="C31" s="9" t="n"/>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>experiences/kayak.jpg</t>
+          <t>experiences/jet-ski.jpg</t>
         </is>
       </c>
       <c r="E31" s="11" t="n"/>
@@ -3097,13 +3240,13 @@
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Paddle</t>
+          <t>Kayak</t>
         </is>
       </c>
       <c r="C32" s="9" t="n"/>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>experiences/paddle.jpg</t>
+          <t>experiences/kayak.jpg</t>
         </is>
       </c>
       <c r="E32" s="11" t="n"/>
@@ -3118,13 +3261,13 @@
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Balade à cheval</t>
+          <t>Paddle</t>
         </is>
       </c>
       <c r="C33" s="9" t="n"/>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>experiences/balade-a-cheval.jpg</t>
+          <t>experiences/paddle.jpg</t>
         </is>
       </c>
       <c r="E33" s="11" t="n"/>
@@ -3139,13 +3282,13 @@
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Excursion en chaloupe (+2 photos)</t>
+          <t>Balade à cheval</t>
         </is>
       </c>
       <c r="C34" s="9" t="n"/>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>experiences/excursion-en-chaloupe.jpg</t>
+          <t>experiences/balade-a-cheval.jpg</t>
         </is>
       </c>
       <c r="E34" s="11" t="n"/>
@@ -3160,13 +3303,13 @@
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>Excursion en pirogue (+2 photos)</t>
+          <t>Excursion en chaloupe (+2 photos)</t>
         </is>
       </c>
       <c r="C35" s="9" t="n"/>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>experiences/excursion-en-pirogue.jpg</t>
+          <t>experiences/excursion-en-chaloupe.jpg</t>
         </is>
       </c>
       <c r="E35" s="11" t="n"/>
@@ -3181,13 +3324,13 @@
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>Bateau de croisière en haute mer</t>
+          <t>Excursion en pirogue (+2 photos)</t>
         </is>
       </c>
       <c r="C36" s="9" t="n"/>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>illustrations/croisiere-en-haute-mer.jpg</t>
+          <t>experiences/excursion-en-pirogue.jpg</t>
         </is>
       </c>
       <c r="E36" s="11" t="n"/>
@@ -3202,13 +3345,13 @@
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>Jacuzzi naturel (+2 photos)</t>
+          <t>Bateau de croisière en haute mer</t>
         </is>
       </c>
       <c r="C37" s="9" t="n"/>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>experiences/jacuzzi-naturel.jpg</t>
+          <t>illustrations/croisiere-en-haute-mer.jpg</t>
         </is>
       </c>
       <c r="E37" s="11" t="n"/>
@@ -3223,13 +3366,13 @@
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>Feu de camp ou feu de plage (+2 photos)</t>
+          <t>Jacuzzi naturel (+2 photos)</t>
         </is>
       </c>
       <c r="C38" s="9" t="n"/>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>experiences/feu-de-plage.jpg</t>
+          <t>experiences/jacuzzi-naturel.jpg</t>
         </is>
       </c>
       <c r="E38" s="11" t="n"/>
@@ -3244,13 +3387,13 @@
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>Séance photo à Kribi (+2 photos)</t>
+          <t>Feu de camp ou feu de plage (+2 photos)</t>
         </is>
       </c>
       <c r="C39" s="9" t="n"/>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>experiences/seance-photo.jpg</t>
+          <t>experiences/feu-de-plage.jpg</t>
         </is>
       </c>
       <c r="E39" s="11" t="n"/>
@@ -3265,13 +3408,13 @@
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>Pique-nique et bivouac en bord de mer (+1 photo)</t>
+          <t>Séance photo à Kribi (+2 photos)</t>
         </is>
       </c>
       <c r="C40" s="9" t="n"/>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>experiences/pique-nique-bivouac.jpg</t>
+          <t>experiences/seance-photo.jpg</t>
         </is>
       </c>
       <c r="E40" s="11" t="n"/>
@@ -3286,52 +3429,52 @@
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>Bouée tractée (+1 photo)</t>
+          <t>Pique-nique en bord de mer (+1 photo)</t>
         </is>
       </c>
       <c r="C41" s="9" t="n"/>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>experiences/bouee-tractee.jpg</t>
+          <t>experiences/pique-nique-bivouac.jpg</t>
         </is>
       </c>
       <c r="E41" s="11" t="n"/>
       <c r="F41" s="11" t="n"/>
       <c r="G41" s="11" t="n"/>
     </row>
-    <row r="42">
-      <c r="A42" s="12" t="inlineStr">
+    <row r="42" ht="80" customHeight="1">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>Tourisme — Activités &amp; Loisirs</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>Bouée tractée (+1 photo)</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="n"/>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>experiences/bouee-tractee.jpg</t>
+        </is>
+      </c>
+      <c r="E42" s="11" t="n"/>
+      <c r="F42" s="11" t="n"/>
+      <c r="G42" s="11" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
         <is>
           <t>Tourisme — Spécialités culinaires</t>
         </is>
       </c>
-      <c r="B42" s="13" t="n"/>
-      <c r="C42" s="13" t="n"/>
-      <c r="D42" s="13" t="n"/>
-      <c r="E42" s="13" t="n"/>
-      <c r="F42" s="13" t="n"/>
-      <c r="G42" s="13" t="n"/>
-    </row>
-    <row r="43" ht="80" customHeight="1">
-      <c r="A43" s="9" t="inlineStr">
-        <is>
-          <t>Tourisme — Spécialités culinaires</t>
-        </is>
-      </c>
-      <c r="B43" s="8" t="inlineStr">
-        <is>
-          <t>Poisson frais ou braisé</t>
-        </is>
-      </c>
-      <c r="C43" s="9" t="n"/>
-      <c r="D43" s="9" t="inlineStr">
-        <is>
-          <t>illustrations/poisson-braise.jpg</t>
-        </is>
-      </c>
-      <c r="E43" s="11" t="n"/>
-      <c r="F43" s="11" t="n"/>
-      <c r="G43" s="11" t="n"/>
+      <c r="B43" s="13" t="n"/>
+      <c r="C43" s="13" t="n"/>
+      <c r="D43" s="13" t="n"/>
+      <c r="E43" s="13" t="n"/>
+      <c r="F43" s="13" t="n"/>
+      <c r="G43" s="13" t="n"/>
     </row>
     <row r="44" ht="80" customHeight="1">
       <c r="A44" s="9" t="inlineStr">
@@ -3341,13 +3484,13 @@
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>Gambas</t>
+          <t>Poisson frais ou braisé</t>
         </is>
       </c>
       <c r="C44" s="9" t="n"/>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>illustrations/gambas.jpg</t>
+          <t>illustrations/poisson-braise.jpg</t>
         </is>
       </c>
       <c r="E44" s="11" t="n"/>
@@ -3362,13 +3505,13 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Crevettes</t>
+          <t>Gambas</t>
         </is>
       </c>
       <c r="C45" s="9" t="n"/>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>illustrations/crevettes.jpg</t>
+          <t>illustrations/gambas.jpg</t>
         </is>
       </c>
       <c r="E45" s="11" t="n"/>
@@ -3383,13 +3526,13 @@
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>Crabe</t>
+          <t>Crevettes</t>
         </is>
       </c>
       <c r="C46" s="9" t="n"/>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>illustrations/crabe.jpg</t>
+          <t>illustrations/crevettes.jpg</t>
         </is>
       </c>
       <c r="E46" s="11" t="n"/>
@@ -3404,13 +3547,13 @@
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>Langouste</t>
+          <t>Crabe</t>
         </is>
       </c>
       <c r="C47" s="9" t="n"/>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>illustrations/langouste.jpg</t>
+          <t>illustrations/crabe.jpg</t>
         </is>
       </c>
       <c r="E47" s="11" t="n"/>
@@ -3425,13 +3568,13 @@
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>Maban, poisson pimenté</t>
+          <t>Langouste</t>
         </is>
       </c>
       <c r="C48" s="9" t="n"/>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>illustrations/maban.jpg</t>
+          <t>illustrations/langouste.jpg</t>
         </is>
       </c>
       <c r="E48" s="11" t="n"/>
@@ -3446,13 +3589,13 @@
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>Noix de coco fraîche à boire</t>
+          <t>Maban, poisson pimenté</t>
         </is>
       </c>
       <c r="C49" s="9" t="n"/>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>illustrations/noix-de-coco.jpg</t>
+          <t>sections/plage-kribi.jpg</t>
         </is>
       </c>
       <c r="E49" s="11" t="n"/>
@@ -3467,13 +3610,13 @@
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>Grillades et barbecue de plage</t>
+          <t>Ebanjea, spécialité batanga</t>
         </is>
       </c>
       <c r="C50" s="9" t="n"/>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>illustrations/grillades-de-plage.jpg</t>
+          <t>sections/plage-kribi.jpg</t>
         </is>
       </c>
       <c r="E50" s="11" t="n"/>
@@ -3488,13 +3631,13 @@
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>Dégustation de fruits de mer en bord de mer</t>
+          <t>Noix de coco fraîche à boire</t>
         </is>
       </c>
       <c r="C51" s="9" t="n"/>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>illustrations/degustation-fruits-de-mer.jpg</t>
+          <t>illustrations/noix-de-coco.jpg</t>
         </is>
       </c>
       <c r="E51" s="11" t="n"/>
@@ -3509,73 +3652,73 @@
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>Expérience de repas local</t>
+          <t>Grillades et barbecue de plage</t>
         </is>
       </c>
       <c r="C52" s="9" t="n"/>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>illustrations/repas-local.jpg</t>
+          <t>illustrations/grillades-de-plage.jpg</t>
         </is>
       </c>
       <c r="E52" s="11" t="n"/>
       <c r="F52" s="11" t="n"/>
       <c r="G52" s="11" t="n"/>
     </row>
-    <row r="53">
-      <c r="A53" s="12" t="inlineStr">
-        <is>
-          <t>Parcours</t>
-        </is>
-      </c>
-      <c r="B53" s="13" t="n"/>
-      <c r="C53" s="13" t="n"/>
-      <c r="D53" s="13" t="n"/>
-      <c r="E53" s="13" t="n"/>
-      <c r="F53" s="13" t="n"/>
-      <c r="G53" s="13" t="n"/>
+    <row r="53" ht="80" customHeight="1">
+      <c r="A53" s="9" t="inlineStr">
+        <is>
+          <t>Tourisme — Spécialités culinaires</t>
+        </is>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>Dégustation de fruits de mer en bord de mer</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="n"/>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>illustrations/degustation-fruits-de-mer.jpg</t>
+        </is>
+      </c>
+      <c r="E53" s="11" t="n"/>
+      <c r="F53" s="11" t="n"/>
+      <c r="G53" s="11" t="n"/>
     </row>
     <row r="54" ht="80" customHeight="1">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t>Parcours</t>
+          <t>Tourisme — Spécialités culinaires</t>
         </is>
       </c>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>L'Essentiel de Kribi</t>
+          <t>Expérience de repas local</t>
         </is>
       </c>
       <c r="C54" s="9" t="n"/>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>experiences/chutes-de-la-lobe.jpg</t>
+          <t>illustrations/repas-local.jpg</t>
         </is>
       </c>
       <c r="E54" s="11" t="n"/>
       <c r="F54" s="11" t="n"/>
       <c r="G54" s="11" t="n"/>
     </row>
-    <row r="55" ht="80" customHeight="1">
-      <c r="A55" s="9" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="12" t="inlineStr">
         <is>
           <t>Parcours</t>
         </is>
       </c>
-      <c r="B55" s="8" t="inlineStr">
-        <is>
-          <t>Kribi Nature &amp; Littoral</t>
-        </is>
-      </c>
-      <c r="C55" s="9" t="n"/>
-      <c r="D55" s="9" t="inlineStr">
-        <is>
-          <t>experiences/chutes-de-la-lobe-2.jpg</t>
-        </is>
-      </c>
-      <c r="E55" s="11" t="n"/>
-      <c r="F55" s="11" t="n"/>
-      <c r="G55" s="11" t="n"/>
+      <c r="B55" s="13" t="n"/>
+      <c r="C55" s="13" t="n"/>
+      <c r="D55" s="13" t="n"/>
+      <c r="E55" s="13" t="n"/>
+      <c r="F55" s="13" t="n"/>
+      <c r="G55" s="13" t="n"/>
     </row>
     <row r="56" ht="80" customHeight="1">
       <c r="A56" s="9" t="inlineStr">
@@ -3585,13 +3728,13 @@
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>Kribi Culture &amp; Patrimoine</t>
+          <t>L'Essentiel de Kribi</t>
         </is>
       </c>
       <c r="C56" s="9" t="n"/>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>experiences/village-mayi.jpg</t>
+          <t>experiences/chutes-de-la-lobe.jpg</t>
         </is>
       </c>
       <c r="E56" s="11" t="n"/>
@@ -3606,13 +3749,13 @@
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>Kribi &amp; Ebodjé</t>
+          <t>Kribi Nature &amp; Littoral</t>
         </is>
       </c>
       <c r="C57" s="9" t="n"/>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>sections/kribi-vue-aerienne.jpg</t>
+          <t>experiences/chutes-de-la-lobe-2.jpg</t>
         </is>
       </c>
       <c r="E57" s="11" t="n"/>
@@ -3627,13 +3770,13 @@
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>Kribi Authentique</t>
+          <t>Kribi Culture &amp; Patrimoine</t>
         </is>
       </c>
       <c r="C58" s="9" t="n"/>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>experiences/campement-bagyeli.jpg</t>
+          <t>experiences/village-mayi.jpg</t>
         </is>
       </c>
       <c r="E58" s="11" t="n"/>
@@ -3648,41 +3791,49 @@
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>Kribi au fil de l'eau</t>
+          <t>Kribi &amp; Ebodjé</t>
         </is>
       </c>
       <c r="C59" s="9" t="n"/>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>experiences/excursion-en-pirogue.jpg</t>
+          <t>sections/kribi-vue-aerienne.jpg</t>
         </is>
       </c>
       <c r="E59" s="11" t="n"/>
       <c r="F59" s="11" t="n"/>
       <c r="G59" s="11" t="n"/>
     </row>
-    <row r="60">
-      <c r="A60" s="12" t="inlineStr">
-        <is>
-          <t>Formules</t>
-        </is>
-      </c>
-      <c r="B60" s="13" t="n"/>
-      <c r="C60" s="13" t="n"/>
-      <c r="D60" s="13" t="n"/>
-      <c r="E60" s="13" t="n"/>
-      <c r="F60" s="13" t="n"/>
-      <c r="G60" s="13" t="n"/>
+    <row r="60" ht="80" customHeight="1">
+      <c r="A60" s="9" t="inlineStr">
+        <is>
+          <t>Parcours</t>
+        </is>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>Kribi Authentique</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="n"/>
+      <c r="D60" s="9" t="inlineStr">
+        <is>
+          <t>experiences/campement-bagyeli.jpg</t>
+        </is>
+      </c>
+      <c r="E60" s="11" t="n"/>
+      <c r="F60" s="11" t="n"/>
+      <c r="G60" s="11" t="n"/>
     </row>
     <row r="61" ht="80" customHeight="1">
       <c r="A61" s="9" t="inlineStr">
         <is>
-          <t>Formules</t>
+          <t>Parcours</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>Formule Découverte</t>
+          <t>Kribi au fil de l'eau</t>
         </is>
       </c>
       <c r="C61" s="9" t="n"/>
@@ -3695,26 +3846,18 @@
       <c r="F61" s="11" t="n"/>
       <c r="G61" s="11" t="n"/>
     </row>
-    <row r="62" ht="80" customHeight="1">
-      <c r="A62" s="9" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="12" t="inlineStr">
         <is>
           <t>Formules</t>
         </is>
       </c>
-      <c r="B62" s="8" t="inlineStr">
-        <is>
-          <t>Formule Évasion</t>
-        </is>
-      </c>
-      <c r="C62" s="9" t="n"/>
-      <c r="D62" s="9" t="inlineStr">
-        <is>
-          <t>experiences/balade-a-cheval.jpg</t>
-        </is>
-      </c>
-      <c r="E62" s="11" t="n"/>
-      <c r="F62" s="11" t="n"/>
-      <c r="G62" s="11" t="n"/>
+      <c r="B62" s="13" t="n"/>
+      <c r="C62" s="13" t="n"/>
+      <c r="D62" s="13" t="n"/>
+      <c r="E62" s="13" t="n"/>
+      <c r="F62" s="13" t="n"/>
+      <c r="G62" s="13" t="n"/>
     </row>
     <row r="63" ht="80" customHeight="1">
       <c r="A63" s="9" t="inlineStr">
@@ -3724,13 +3867,13 @@
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>Formule Aventure</t>
+          <t>Formule Découverte</t>
         </is>
       </c>
       <c r="C63" s="9" t="n"/>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>experiences/quad.jpg</t>
+          <t>experiences/excursion-en-pirogue.jpg</t>
         </is>
       </c>
       <c r="E63" s="11" t="n"/>
@@ -3745,73 +3888,73 @@
       </c>
       <c r="B64" s="8" t="inlineStr">
         <is>
-          <t>Formule Premium</t>
+          <t>Formule Évasion</t>
         </is>
       </c>
       <c r="C64" s="9" t="n"/>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>illustrations/croisiere-en-haute-mer.jpg</t>
+          <t>experiences/balade-a-cheval.jpg</t>
         </is>
       </c>
       <c r="E64" s="11" t="n"/>
       <c r="F64" s="11" t="n"/>
       <c r="G64" s="11" t="n"/>
     </row>
-    <row r="65">
-      <c r="A65" s="12" t="inlineStr">
-        <is>
-          <t>Hébergements par budget</t>
-        </is>
-      </c>
-      <c r="B65" s="13" t="n"/>
-      <c r="C65" s="13" t="n"/>
-      <c r="D65" s="13" t="n"/>
-      <c r="E65" s="13" t="n"/>
-      <c r="F65" s="13" t="n"/>
-      <c r="G65" s="13" t="n"/>
+    <row r="65" ht="80" customHeight="1">
+      <c r="A65" s="9" t="inlineStr">
+        <is>
+          <t>Formules</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>Formule Aventure</t>
+        </is>
+      </c>
+      <c r="C65" s="9" t="n"/>
+      <c r="D65" s="9" t="inlineStr">
+        <is>
+          <t>experiences/quad.jpg</t>
+        </is>
+      </c>
+      <c r="E65" s="11" t="n"/>
+      <c r="F65" s="11" t="n"/>
+      <c r="G65" s="11" t="n"/>
     </row>
     <row r="66" ht="80" customHeight="1">
       <c r="A66" s="9" t="inlineStr">
         <is>
-          <t>Hébergements par budget</t>
+          <t>Formules</t>
         </is>
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>Chambre, à partir de 15 000 FCFA la nuit</t>
+          <t>Formule Premium</t>
         </is>
       </c>
       <c r="C66" s="9" t="n"/>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>illustrations/chambre-15000.jpg</t>
+          <t>illustrations/croisiere-en-haute-mer.jpg</t>
         </is>
       </c>
       <c r="E66" s="11" t="n"/>
       <c r="F66" s="11" t="n"/>
       <c r="G66" s="11" t="n"/>
     </row>
-    <row r="67" ht="80" customHeight="1">
-      <c r="A67" s="9" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="12" t="inlineStr">
         <is>
           <t>Hébergements par budget</t>
         </is>
       </c>
-      <c r="B67" s="8" t="inlineStr">
-        <is>
-          <t>Studio, à partir de 30 000 FCFA la nuit</t>
-        </is>
-      </c>
-      <c r="C67" s="9" t="n"/>
-      <c r="D67" s="9" t="inlineStr">
-        <is>
-          <t>illustrations/studio-30000.jpg</t>
-        </is>
-      </c>
-      <c r="E67" s="11" t="n"/>
-      <c r="F67" s="11" t="n"/>
-      <c r="G67" s="11" t="n"/>
+      <c r="B67" s="13" t="n"/>
+      <c r="C67" s="13" t="n"/>
+      <c r="D67" s="13" t="n"/>
+      <c r="E67" s="13" t="n"/>
+      <c r="F67" s="13" t="n"/>
+      <c r="G67" s="13" t="n"/>
     </row>
     <row r="68" ht="80" customHeight="1">
       <c r="A68" s="9" t="inlineStr">
@@ -3821,13 +3964,13 @@
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>Appartement, à partir de 35 000 FCFA la nuit</t>
+          <t>Chambre, à partir de 15 000 FCFA la nuit</t>
         </is>
       </c>
       <c r="C68" s="9" t="n"/>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>illustrations/appartement-35000.jpg</t>
+          <t>illustrations/chambre-15000.jpg</t>
         </is>
       </c>
       <c r="E68" s="11" t="n"/>
@@ -3842,13 +3985,13 @@
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>Appartement, à partir de 50 000 FCFA la nuit</t>
+          <t>Studio, à partir de 30 000 FCFA la nuit</t>
         </is>
       </c>
       <c r="C69" s="9" t="n"/>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>illustrations/appartement-50000.jpg</t>
+          <t>illustrations/studio-30000.jpg</t>
         </is>
       </c>
       <c r="E69" s="11" t="n"/>
@@ -3863,13 +4006,13 @@
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t>Appartement, à partir de 100 000 FCFA la nuit</t>
+          <t>Appartement, à partir de 35 000 FCFA la nuit</t>
         </is>
       </c>
       <c r="C70" s="9" t="n"/>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>illustrations/appartement-100000.jpg</t>
+          <t>illustrations/appartement-35000.jpg</t>
         </is>
       </c>
       <c r="E70" s="11" t="n"/>
@@ -3884,73 +4027,73 @@
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>Villa, à partir de 150 000 FCFA la nuit</t>
+          <t>Appartement, à partir de 50 000 FCFA la nuit</t>
         </is>
       </c>
       <c r="C71" s="9" t="n"/>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>illustrations/villa-150000.jpg</t>
+          <t>illustrations/appartement-50000.jpg</t>
         </is>
       </c>
       <c r="E71" s="11" t="n"/>
       <c r="F71" s="11" t="n"/>
       <c r="G71" s="11" t="n"/>
     </row>
-    <row r="72">
-      <c r="A72" s="12" t="inlineStr">
-        <is>
-          <t>Mobilité TKS®</t>
-        </is>
-      </c>
-      <c r="B72" s="13" t="n"/>
-      <c r="C72" s="13" t="n"/>
-      <c r="D72" s="13" t="n"/>
-      <c r="E72" s="13" t="n"/>
-      <c r="F72" s="13" t="n"/>
-      <c r="G72" s="13" t="n"/>
+    <row r="72" ht="80" customHeight="1">
+      <c r="A72" s="9" t="inlineStr">
+        <is>
+          <t>Hébergements par budget</t>
+        </is>
+      </c>
+      <c r="B72" s="8" t="inlineStr">
+        <is>
+          <t>Appartement, à partir de 100 000 FCFA la nuit</t>
+        </is>
+      </c>
+      <c r="C72" s="9" t="n"/>
+      <c r="D72" s="9" t="inlineStr">
+        <is>
+          <t>illustrations/appartement-100000.jpg</t>
+        </is>
+      </c>
+      <c r="E72" s="11" t="n"/>
+      <c r="F72" s="11" t="n"/>
+      <c r="G72" s="11" t="n"/>
     </row>
     <row r="73" ht="80" customHeight="1">
       <c r="A73" s="9" t="inlineStr">
         <is>
-          <t>Mobilité TKS®</t>
+          <t>Hébergements par budget</t>
         </is>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>Luxe (+1 photo)</t>
+          <t>Villa, à partir de 150 000 FCFA la nuit</t>
         </is>
       </c>
       <c r="C73" s="9" t="n"/>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>mobility/luxe.jpg</t>
+          <t>illustrations/villa-150000.jpg</t>
         </is>
       </c>
       <c r="E73" s="11" t="n"/>
       <c r="F73" s="11" t="n"/>
       <c r="G73" s="11" t="n"/>
     </row>
-    <row r="74" ht="80" customHeight="1">
-      <c r="A74" s="9" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="12" t="inlineStr">
         <is>
           <t>Mobilité TKS®</t>
         </is>
       </c>
-      <c r="B74" s="8" t="inlineStr">
-        <is>
-          <t>Premium (+1 photo)</t>
-        </is>
-      </c>
-      <c r="C74" s="9" t="n"/>
-      <c r="D74" s="9" t="inlineStr">
-        <is>
-          <t>mobility/premium.jpg</t>
-        </is>
-      </c>
-      <c r="E74" s="11" t="n"/>
-      <c r="F74" s="11" t="n"/>
-      <c r="G74" s="11" t="n"/>
+      <c r="B74" s="13" t="n"/>
+      <c r="C74" s="13" t="n"/>
+      <c r="D74" s="13" t="n"/>
+      <c r="E74" s="13" t="n"/>
+      <c r="F74" s="13" t="n"/>
+      <c r="G74" s="13" t="n"/>
     </row>
     <row r="75" ht="80" customHeight="1">
       <c r="A75" s="9" t="inlineStr">
@@ -3960,13 +4103,13 @@
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>Yaris</t>
+          <t>Luxe (+1 photo)</t>
         </is>
       </c>
       <c r="C75" s="9" t="n"/>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>mobility/yaris.jpg</t>
+          <t>mobility/luxe.jpg</t>
         </is>
       </c>
       <c r="E75" s="11" t="n"/>
@@ -3981,13 +4124,13 @@
       </c>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>Location avec chauffeur</t>
+          <t>Premium (+1 photo)</t>
         </is>
       </c>
       <c r="C76" s="9" t="n"/>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>mobility/luxe-2.jpg</t>
+          <t>mobility/premium.jpg</t>
         </is>
       </c>
       <c r="E76" s="11" t="n"/>
@@ -4002,13 +4145,13 @@
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>Transferts</t>
+          <t>Yaris</t>
         </is>
       </c>
       <c r="C77" s="9" t="n"/>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>mobility/premium-2.jpg</t>
+          <t>mobility/yaris.jpg</t>
         </is>
       </c>
       <c r="E77" s="11" t="n"/>
@@ -4023,13 +4166,13 @@
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>Chauffeur privé</t>
+          <t>Location avec chauffeur</t>
         </is>
       </c>
       <c r="C78" s="9" t="n"/>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>mobility/luxe.jpg</t>
+          <t>mobility/luxe-2.jpg</t>
         </is>
       </c>
       <c r="E78" s="11" t="n"/>
@@ -4044,22 +4187,64 @@
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>Prestations professionnelles</t>
+          <t>Transferts</t>
         </is>
       </c>
       <c r="C79" s="9" t="n"/>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>mobility/premium.jpg</t>
+          <t>mobility/premium-2.jpg</t>
         </is>
       </c>
       <c r="E79" s="11" t="n"/>
       <c r="F79" s="11" t="n"/>
       <c r="G79" s="11" t="n"/>
     </row>
+    <row r="80" ht="80" customHeight="1">
+      <c r="A80" s="9" t="inlineStr">
+        <is>
+          <t>Mobilité TKS®</t>
+        </is>
+      </c>
+      <c r="B80" s="8" t="inlineStr">
+        <is>
+          <t>Chauffeur privé</t>
+        </is>
+      </c>
+      <c r="C80" s="9" t="n"/>
+      <c r="D80" s="9" t="inlineStr">
+        <is>
+          <t>mobility/luxe.jpg</t>
+        </is>
+      </c>
+      <c r="E80" s="11" t="n"/>
+      <c r="F80" s="11" t="n"/>
+      <c r="G80" s="11" t="n"/>
+    </row>
+    <row r="81" ht="80" customHeight="1">
+      <c r="A81" s="9" t="inlineStr">
+        <is>
+          <t>Mobilité TKS®</t>
+        </is>
+      </c>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>Prestations professionnelles</t>
+        </is>
+      </c>
+      <c r="C81" s="9" t="n"/>
+      <c r="D81" s="9" t="inlineStr">
+        <is>
+          <t>mobility/premium.jpg</t>
+        </is>
+      </c>
+      <c r="E81" s="11" t="n"/>
+      <c r="F81" s="11" t="n"/>
+      <c r="G81" s="11" t="n"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="E5:E80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E5:E82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Garder,Changer,Garder et ajouter des photos"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>